<commit_message>
Ya certifica de manera sola, solo falta guardar los resultados en un excel y mejorar LA VISTA
</commit_message>
<xml_diff>
--- a/datos/Fichas.xlsx
+++ b/datos/Fichas.xlsx
@@ -339,7 +339,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -349,21 +349,11 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>3473168</v>
+        <v>3485326</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>3473180</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3485326</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5">
         <v>3510030</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ya con version en TKINTER
</commit_message>
<xml_diff>
--- a/datos/Fichas.xlsx
+++ b/datos/Fichas.xlsx
@@ -349,12 +349,12 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>3485326</v>
+        <v>3568809</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>3510030</v>
+        <v>3568083</v>
       </c>
     </row>
   </sheetData>

</xml_diff>